<commit_message>
-> Einfügen des Screenshorts -> auftrags_manager.py haben wir die eine Funktion geschreiben das daten in die SQL einsetzt -> nächster schrit die html bauen und dazu noch in eine neue route seite die logik zu diese Funktion schreiben.
</commit_message>
<xml_diff>
--- a/Mitarbeiter/Alle_Bestaende.xlsx
+++ b/Mitarbeiter/Alle_Bestaende.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>5000</v>
+        <v>4500</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -953,6 +953,39 @@
       <c r="G16" t="inlineStr">
         <is>
           <t>Hamburg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DE309012</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Cement säcke</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>cement</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Lemgo</t>
         </is>
       </c>
     </row>

</xml_diff>